<commit_message>
Etapa 3, paso 2: outfits vestibles de Polyvore + tallas 41/42
- src/modelo_fly/polyvore.py: filtrar_outfits y motivo_invalido. Regla: un vestido solo, o
  abajo + 1-2 arriba; exactamente un calzado; como mucho un exterior; bolso, accesorio y
  joyería libres. Se descartan outfits duplicados (mismos productos).
- 00_polyvore_descarga: sección del paso 2. Quedan 15 012 de 21 889 outfits
  (4 172 con vestido, 10 840 arriba + abajo); se guarda polyvore_outfits.csv con el motivo.
- Catálogo propio: tallas de ropa 41 -> XXL y 42 -> XXXL.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/revision/catalogo_propio_revision.xlsx
+++ b/data/revision/catalogo_propio_revision.xlsx
@@ -816,7 +816,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>XXL</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -1256,7 +1256,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>XXXL</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>XXXL</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -2906,7 +2906,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>XXXL</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -3566,7 +3566,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>XXXL</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -3896,7 +3896,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>XXL</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -4336,7 +4336,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>XXXL</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -4446,7 +4446,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>XXL</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -4886,7 +4886,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>XXXL</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -5216,7 +5216,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>XXXL</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -5326,7 +5326,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>XXL</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -5876,7 +5876,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>XXXL</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -6206,7 +6206,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>XXXL</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -6426,7 +6426,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>XXL</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -6976,7 +6976,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>XXL</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -7086,7 +7086,7 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>XXL</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -7196,7 +7196,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>XXL</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -8626,7 +8626,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>XXXL</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -9726,7 +9726,7 @@
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>XXL</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
@@ -9836,7 +9836,7 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>XXXL</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -12366,7 +12366,7 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>XXXL</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
@@ -12586,7 +12586,7 @@
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>XXL</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
@@ -17936,7 +17936,7 @@
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>XXXL</t>
         </is>
       </c>
       <c r="G160" t="inlineStr">
@@ -19568,7 +19568,7 @@
       </c>
       <c r="F176" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>XXXL</t>
         </is>
       </c>
       <c r="G176" t="inlineStr">
@@ -19772,7 +19772,7 @@
       </c>
       <c r="F178" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>XXXL</t>
         </is>
       </c>
       <c r="G178" t="inlineStr">
@@ -20690,7 +20690,7 @@
       </c>
       <c r="F187" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>XXXL</t>
         </is>
       </c>
       <c r="G187" t="inlineStr">
@@ -20894,7 +20894,7 @@
       </c>
       <c r="F189" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>XXL</t>
         </is>
       </c>
       <c r="G189" t="inlineStr">
@@ -21506,7 +21506,7 @@
       </c>
       <c r="F195" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>XXL</t>
         </is>
       </c>
       <c r="G195" t="inlineStr">
@@ -21710,7 +21710,7 @@
       </c>
       <c r="F197" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>XXXL</t>
         </is>
       </c>
       <c r="G197" t="inlineStr">
@@ -22220,7 +22220,7 @@
       </c>
       <c r="F202" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>XXL</t>
         </is>
       </c>
       <c r="G202" t="inlineStr">
@@ -22424,7 +22424,7 @@
       </c>
       <c r="F204" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>XXXL</t>
         </is>
       </c>
       <c r="G204" t="inlineStr">
@@ -23240,7 +23240,7 @@
       </c>
       <c r="F212" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>XXL</t>
         </is>
       </c>
       <c r="G212" t="inlineStr">
@@ -24566,7 +24566,7 @@
       </c>
       <c r="F225" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>XXL</t>
         </is>
       </c>
       <c r="G225" t="inlineStr">
@@ -25280,7 +25280,7 @@
       </c>
       <c r="F232" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>XXL</t>
         </is>
       </c>
       <c r="G232" t="inlineStr">
@@ -26402,7 +26402,7 @@
       </c>
       <c r="F243" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>XXXL</t>
         </is>
       </c>
       <c r="G243" t="inlineStr">
@@ -26810,7 +26810,7 @@
       </c>
       <c r="F247" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>XXXL</t>
         </is>
       </c>
       <c r="G247" t="inlineStr">
@@ -27422,7 +27422,7 @@
       </c>
       <c r="F253" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>XXL</t>
         </is>
       </c>
       <c r="G253" t="inlineStr">
@@ -27626,7 +27626,7 @@
       </c>
       <c r="F255" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>XXXL</t>
         </is>
       </c>
       <c r="G255" t="inlineStr">
@@ -27932,7 +27932,7 @@
       </c>
       <c r="F258" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>XXXL</t>
         </is>
       </c>
       <c r="G258" t="inlineStr">
@@ -29054,7 +29054,7 @@
       </c>
       <c r="F269" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>XXXL</t>
         </is>
       </c>
       <c r="G269" t="inlineStr">
@@ -29360,7 +29360,7 @@
       </c>
       <c r="F272" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>XXL</t>
         </is>
       </c>
       <c r="G272" t="inlineStr">
@@ -29768,7 +29768,7 @@
       </c>
       <c r="F276" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>XXXL</t>
         </is>
       </c>
       <c r="G276" t="inlineStr">
@@ -30074,7 +30074,7 @@
       </c>
       <c r="F279" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>XXXL</t>
         </is>
       </c>
       <c r="G279" t="inlineStr">
@@ -30380,7 +30380,7 @@
       </c>
       <c r="F282" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>XXXL</t>
         </is>
       </c>
       <c r="G282" t="inlineStr">
@@ -30686,7 +30686,7 @@
       </c>
       <c r="F285" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>XXXL</t>
         </is>
       </c>
       <c r="G285" t="inlineStr">
@@ -30890,7 +30890,7 @@
       </c>
       <c r="F287" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>XXL</t>
         </is>
       </c>
       <c r="G287" t="inlineStr">
@@ -30992,7 +30992,7 @@
       </c>
       <c r="F288" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>XXXL</t>
         </is>
       </c>
       <c r="G288" t="inlineStr">
@@ -31094,7 +31094,7 @@
       </c>
       <c r="F289" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>XXL</t>
         </is>
       </c>
       <c r="G289" t="inlineStr">
@@ -31502,7 +31502,7 @@
       </c>
       <c r="F293" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>XXL</t>
         </is>
       </c>
       <c r="G293" t="inlineStr">
@@ -32930,7 +32930,7 @@
       </c>
       <c r="F307" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>XXL</t>
         </is>
       </c>
       <c r="G307" t="inlineStr">
@@ -34052,7 +34052,7 @@
       </c>
       <c r="F318" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>XXL</t>
         </is>
       </c>
       <c r="G318" t="inlineStr">
@@ -34460,7 +34460,7 @@
       </c>
       <c r="F322" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>XXL</t>
         </is>
       </c>
       <c r="G322" t="inlineStr">
@@ -35174,7 +35174,7 @@
       </c>
       <c r="F329" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>XXL</t>
         </is>
       </c>
       <c r="G329" t="inlineStr">
@@ -35582,7 +35582,7 @@
       </c>
       <c r="F333" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>XXXL</t>
         </is>
       </c>
       <c r="G333" t="inlineStr">
@@ -37010,7 +37010,7 @@
       </c>
       <c r="F347" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>XXL</t>
         </is>
       </c>
       <c r="G347" t="inlineStr">
@@ -39764,7 +39764,7 @@
       </c>
       <c r="F374" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>XXL</t>
         </is>
       </c>
       <c r="G374" t="inlineStr">
@@ -42110,7 +42110,7 @@
       </c>
       <c r="F397" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>XXL</t>
         </is>
       </c>
       <c r="G397" t="inlineStr">
@@ -42416,7 +42416,7 @@
       </c>
       <c r="F400" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>XXL</t>
         </is>
       </c>
       <c r="G400" t="inlineStr">
@@ -42518,7 +42518,7 @@
       </c>
       <c r="F401" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>XXXL</t>
         </is>
       </c>
       <c r="G401" t="inlineStr">
@@ -45476,7 +45476,7 @@
       </c>
       <c r="F430" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>XXL</t>
         </is>
       </c>
       <c r="G430" t="inlineStr">
@@ -45680,7 +45680,7 @@
       </c>
       <c r="F432" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>XXXL</t>
         </is>
       </c>
       <c r="G432" t="inlineStr">
@@ -45986,7 +45986,7 @@
       </c>
       <c r="F435" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>XXL</t>
         </is>
       </c>
       <c r="G435" t="inlineStr">
@@ -47006,7 +47006,7 @@
       </c>
       <c r="F445" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>XXXL</t>
         </is>
       </c>
       <c r="G445" t="inlineStr">
@@ -48128,7 +48128,7 @@
       </c>
       <c r="F456" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>XXXL</t>
         </is>
       </c>
       <c r="G456" t="inlineStr">
@@ -48332,7 +48332,7 @@
       </c>
       <c r="F458" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>XXL</t>
         </is>
       </c>
       <c r="G458" t="inlineStr">
@@ -48740,7 +48740,7 @@
       </c>
       <c r="F462" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>XXXL</t>
         </is>
       </c>
       <c r="G462" t="inlineStr">
@@ -49454,7 +49454,7 @@
       </c>
       <c r="F469" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>XXXL</t>
         </is>
       </c>
       <c r="G469" t="inlineStr">
@@ -49862,7 +49862,7 @@
       </c>
       <c r="F473" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>XXXL</t>
         </is>
       </c>
       <c r="G473" t="inlineStr">
@@ -50780,7 +50780,7 @@
       </c>
       <c r="F482" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>XXL</t>
         </is>
       </c>
       <c r="G482" t="inlineStr">
@@ -51188,7 +51188,7 @@
       </c>
       <c r="F486" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>XXXL</t>
         </is>
       </c>
       <c r="G486" t="inlineStr">
@@ -52004,7 +52004,7 @@
       </c>
       <c r="F494" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>XXXL</t>
         </is>
       </c>
       <c r="G494" t="inlineStr">

</xml_diff>